<commit_message>
fix(e5): align stage periods with signed attestations + PKBA C1
Apply corrections from independent GPT-5 audit before Cyclades submission:

- Reciproq period: 22/04/2025 → 30/05/2025 (matches signed attestation,
  was 01/04 → 31/05)
- Hop Hop Immo period: 05/01/2026 → 13/02/2026 (matches signed attestation,
  was "Janvier 2026 — en cours")
- Add legal entity name "LES CLES DU NEUF" alongside Hop Hop Immo brand
  to match the signature on the attestation
- Add candidate number 02248411067 to dossier and Annexe VI-1 xlsx
- Add C1 (Gérer le patrimoine informatique) to PKBA in projects.ts to
  align portfolio web tableau with the dossier PDF/xlsx
</commit_message>
<xml_diff>
--- a/dossier-e5/Annexe-VI-1-tableau-synthese.xlsx
+++ b/dossier-e5/Annexe-VI-1-tableau-synthese.xlsx
@@ -1227,7 +1227,7 @@
       <c r="E3" s="50" t="n"/>
       <c r="F3" s="51" t="inlineStr">
         <is>
-          <t>N° candidat : (à compléter)</t>
+          <t>N° candidat : 02248411067</t>
         </is>
       </c>
       <c r="G3" s="49" t="n"/>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B20" s="62" t="inlineStr">
         <is>
-          <t>01/04/2025 → 31/05/2025</t>
+          <t>22/04/2025 → 30/05/2025</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr"/>
@@ -1757,13 +1757,13 @@
     <row r="30" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Hop Hop Immo — Stage ingénieur logiciel (convention BTS SIO, prolongation alternance 09/2026). Hoppy : assistant immobilier vocal IA (ElevenLabs + LLM, base 28000+ annonces, 24/7). Agents IA marketing. Refonte SEO homepage Next.js (trafic organique x3 en 3 mois, Lighthouse &gt;95).
+          <t>Hop Hop Immo / LES CLES DU NEUF — Stage ingénieur logiciel (convention BTS SIO ; alternance prévue 09/2026). Hoppy : assistant immobilier vocal IA (ElevenLabs + LLM, base 28000+ annonces, 24/7). Agents IA marketing. Refonte SEO homepage Next.js (trafic organique x3 en 3 mois, Lighthouse &gt;95).
 Productions : Hoppy en production (https://hophopimmo.com), agents IA marketing, refonte SEO documentée.</t>
         </is>
       </c>
       <c r="B30" s="62" t="inlineStr">
         <is>
-          <t>01/01/2026 → 06/2026</t>
+          <t>05/01/2026 → 13/02/2026</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr"/>

</xml_diff>